<commit_message>
auto: reporte semana 2026-10-19 → 2026-10-25
</commit_message>
<xml_diff>
--- a/latest-events.xlsx
+++ b/latest-events.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,7 +422,7 @@
         <v>6618</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-10-13 08:47:03</v>
+        <v>2026-10-19 08:46:50</v>
       </c>
       <c r="D2" t="str">
         <v>NO</v>
@@ -436,7 +436,7 @@
         <v>6617</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-10-14 17:43:07</v>
+        <v>2026-10-20 13:27:19</v>
       </c>
       <c r="D3" t="str">
         <v>NO</v>
@@ -450,7 +450,7 @@
         <v>6616</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-10-12 09:44:37</v>
+        <v>2026-10-19 10:28:08</v>
       </c>
       <c r="D4" t="str">
         <v>NO</v>
@@ -464,10 +464,10 @@
         <v>6608</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-10-12 21:34:09</v>
+        <v>2026-10-19 08:35:10</v>
       </c>
       <c r="D5" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="6">
@@ -478,7 +478,7 @@
         <v>6609</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-10-13 10:19:11</v>
+        <v>2026-10-19 10:21:20</v>
       </c>
       <c r="D6" t="str">
         <v>NO</v>
@@ -492,7 +492,7 @@
         <v>6620</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-10-13 11:14:46</v>
+        <v>2026-10-19 11:34:04</v>
       </c>
       <c r="D7" t="str">
         <v>NO</v>
@@ -506,10 +506,10 @@
         <v>6583</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-10-14 03:11:25</v>
+        <v>2026-10-19 12:08:07</v>
       </c>
       <c r="D8" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="9">
@@ -520,7 +520,7 @@
         <v>6593</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-10-12 15:41:34</v>
+        <v>2026-10-19 12:48:15</v>
       </c>
       <c r="D9" t="str">
         <v>NO</v>
@@ -534,10 +534,10 @@
         <v>6597</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-10-12 10:24:35</v>
+        <v>2026-10-19 06:05:40</v>
       </c>
       <c r="D10" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
     </row>
     <row r="11">
@@ -548,7 +548,7 @@
         <v>6598</v>
       </c>
       <c r="C11" t="str">
-        <v>2026-10-12 15:25:43</v>
+        <v>2026-10-19 10:01:46</v>
       </c>
       <c r="D11" t="str">
         <v>NO</v>
@@ -562,10 +562,10 @@
         <v>6586</v>
       </c>
       <c r="C12" t="str">
-        <v>2026-10-13 20:51:31</v>
+        <v>2026-10-19 15:30:08</v>
       </c>
       <c r="D12" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="13">
@@ -576,7 +576,7 @@
         <v>6604</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-10-14 14:36:05</v>
+        <v>2026-10-19 12:50:29</v>
       </c>
       <c r="D13" t="str">
         <v>NO</v>
@@ -590,7 +590,7 @@
         <v>6601</v>
       </c>
       <c r="C14" t="str">
-        <v>2026-10-14 13:51:40</v>
+        <v>2026-10-19 12:22:24</v>
       </c>
       <c r="D14" t="str">
         <v>NO</v>
@@ -604,10 +604,10 @@
         <v>6606</v>
       </c>
       <c r="C15" t="str">
-        <v>2026-10-12 04:00:20</v>
+        <v>2026-10-19 09:37:59</v>
       </c>
       <c r="D15" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="16">
@@ -618,7 +618,7 @@
         <v>6580</v>
       </c>
       <c r="C16" t="str">
-        <v>2026-10-13 12:17:08</v>
+        <v>2026-10-19 10:59:28</v>
       </c>
       <c r="D16" t="str">
         <v>NO</v>
@@ -632,7 +632,7 @@
         <v>6594</v>
       </c>
       <c r="C17" t="str">
-        <v>2026-10-13 11:04:07</v>
+        <v>2026-10-19 11:08:29</v>
       </c>
       <c r="D17" t="str">
         <v>NO</v>
@@ -646,7 +646,7 @@
         <v>6605</v>
       </c>
       <c r="C18" t="str">
-        <v>2026-10-13 11:07:11</v>
+        <v>2026-10-19 10:58:31</v>
       </c>
       <c r="D18" t="str">
         <v>NO</v>
@@ -660,7 +660,7 @@
         <v>6603</v>
       </c>
       <c r="C19" t="str">
-        <v>2026-10-13 09:56:59</v>
+        <v>2026-10-19 11:38:11</v>
       </c>
       <c r="D19" t="str">
         <v>NO</v>
@@ -674,7 +674,7 @@
         <v>6607</v>
       </c>
       <c r="C20" t="str">
-        <v>2026-10-12 05:33:27</v>
+        <v>2026-10-19 04:56:11</v>
       </c>
       <c r="D20" t="str">
         <v>SI</v>
@@ -688,7 +688,7 @@
         <v>6602</v>
       </c>
       <c r="C21" t="str">
-        <v>2026-10-13 14:11:34</v>
+        <v>2026-10-19 09:23:45</v>
       </c>
       <c r="D21" t="str">
         <v>NO</v>
@@ -702,7 +702,7 @@
         <v>6612</v>
       </c>
       <c r="C22" t="str">
-        <v>2026-10-13 11:09:46</v>
+        <v>2026-10-19 10:52:27</v>
       </c>
       <c r="D22" t="str">
         <v>NO</v>
@@ -716,7 +716,7 @@
         <v>6599</v>
       </c>
       <c r="C23" t="str">
-        <v>2026-10-13 10:49:25</v>
+        <v>2026-10-19 10:48:03</v>
       </c>
       <c r="D23" t="str">
         <v>NO</v>
@@ -724,13 +724,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>GV FOSERO SJHW-18 V OLIVARES</v>
+        <v>GV FORD BU-9781 V OLIVARES</v>
       </c>
       <c r="B24">
-        <v>6592</v>
+        <v>6621</v>
       </c>
       <c r="C24" t="str">
-        <v>2026-10-13 07:12:16</v>
+        <v>2026-10-19 18:02:11</v>
       </c>
       <c r="D24" t="str">
         <v>NO</v>
@@ -738,13 +738,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>GV PEUGEOT THJY-73 J PONCE</v>
+        <v>GV FOSERO SJHW-18 V OLIVARES</v>
       </c>
       <c r="B25">
-        <v>6595</v>
+        <v>6592</v>
       </c>
       <c r="C25" t="str">
-        <v>2026-10-13 10:02:35</v>
+        <v>2026-10-19 07:08:35</v>
       </c>
       <c r="D25" t="str">
         <v>NO</v>
@@ -752,13 +752,13 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>GV SHDV-50 C CARDENAS</v>
+        <v>GV PEUGEOT THJY-73 J PONCE</v>
       </c>
       <c r="B26">
-        <v>6585</v>
+        <v>6595</v>
       </c>
       <c r="C26" t="str">
-        <v>2026-10-13 10:17:31</v>
+        <v>2026-10-19 09:55:28</v>
       </c>
       <c r="D26" t="str">
         <v>NO</v>
@@ -766,13 +766,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>GV SHLC-74 B MIRANDA</v>
+        <v>GV SHDV-50 C CARDENAS</v>
       </c>
       <c r="B27">
-        <v>6588</v>
+        <v>6585</v>
       </c>
       <c r="C27" t="str">
-        <v>2026-10-13 11:01:56</v>
+        <v>2026-10-19 10:17:23</v>
       </c>
       <c r="D27" t="str">
         <v>NO</v>
@@ -780,13 +780,13 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>GV TDKV-88 L CORDERO</v>
+        <v>GV SHLC-74 B MIRANDA</v>
       </c>
       <c r="B28">
-        <v>6587</v>
+        <v>6588</v>
       </c>
       <c r="C28" t="str">
-        <v>2026-10-13 10:24:10</v>
+        <v>2026-10-19 11:02:21</v>
       </c>
       <c r="D28" t="str">
         <v>NO</v>
@@ -794,13 +794,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>GV TDLD-98 J PACHECHO</v>
+        <v>GV TDKV-88 L CORDERO</v>
       </c>
       <c r="B29">
-        <v>6582</v>
+        <v>6587</v>
       </c>
       <c r="C29" t="str">
-        <v>2026-10-13 14:12:20</v>
+        <v>2026-10-19 10:25:15</v>
       </c>
       <c r="D29" t="str">
         <v>NO</v>
@@ -808,13 +808,13 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>GV TM5 RXXG-15 E CABANILLA</v>
+        <v>GV TDLD-98 J PACHECHO</v>
       </c>
       <c r="B30">
-        <v>6589</v>
+        <v>6582</v>
       </c>
       <c r="C30" t="str">
-        <v>2026-10-13 12:04:37</v>
+        <v>2026-10-19 10:58:12</v>
       </c>
       <c r="D30" t="str">
         <v>NO</v>
@@ -822,13 +822,13 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>GV TM5 TDLD-46 M MARTINEZ</v>
+        <v>GV TM5 RXXG-15 E CABANILLA</v>
       </c>
       <c r="B31">
-        <v>6596</v>
+        <v>6589</v>
       </c>
       <c r="C31" t="str">
-        <v>2026-10-13 11:16:29</v>
+        <v>2026-10-19 13:21:06</v>
       </c>
       <c r="D31" t="str">
         <v>NO</v>
@@ -836,42 +836,56 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>GV TOLVA SPGW-29 V OLIVARES</v>
+        <v>GV TM5 TDLD-46 M MARTINEZ</v>
       </c>
       <c r="B32">
-        <v>6619</v>
+        <v>6596</v>
       </c>
       <c r="C32" t="str">
-        <v>2026-10-13 20:35:48</v>
+        <v>2026-10-19 14:16:34</v>
       </c>
       <c r="D32" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
+        <v>GV TOLVA SPGW-29 V OLIVARES</v>
+      </c>
+      <c r="B33">
+        <v>6619</v>
+      </c>
+      <c r="C33" t="str">
+        <v>2026-10-19 13:40:11</v>
+      </c>
+      <c r="D33" t="str">
+        <v>NO</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
         <v>JAC  LYTS-17 G GALEA</v>
       </c>
-      <c r="B33">
+      <c r="B34">
         <v>6614</v>
       </c>
-      <c r="C33" t="str">
-        <v>2026-10-13 08:47:41</v>
-      </c>
-      <c r="D33" t="str">
+      <c r="C34" t="str">
+        <v>2026-10-19 08:49:14</v>
+      </c>
+      <c r="D34" t="str">
         <v>NO</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D34"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -889,10 +903,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>GC TM5-RXXG-13 D SILVA</v>
+        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
       </c>
       <c r="B2">
-        <v>6608</v>
+        <v>6597</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -903,10 +917,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>GLP ALJIBE SJHW-20</v>
+        <v>GP DONGFENG DF6-RXDL-60</v>
       </c>
       <c r="B3">
-        <v>6583</v>
+        <v>6607</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -917,66 +931,66 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>GLP SHLC-75 L FONSECA</v>
+        <v>DONGFENG DF6 SRSR-97</v>
       </c>
       <c r="B4">
-        <v>6586</v>
+        <v>6618</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>GLP SKDX-44 V VIAL</v>
+        <v>GC MAXUS PCRF-25 TERRENO</v>
       </c>
       <c r="B5">
-        <v>6606</v>
+        <v>6617</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>GP DONGFENG DF6-RXDL-60</v>
+        <v>GC MAXUS PKFF-65 G VICENCIO</v>
       </c>
       <c r="B6">
-        <v>6607</v>
+        <v>6616</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>GV TOLVA SPGW-29 V OLIVARES</v>
+        <v>GC TM5-RXXG-13 D SILVA</v>
       </c>
       <c r="B7">
-        <v>6619</v>
+        <v>6608</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>DONGFENG DF6 SRSR-97</v>
+        <v>GC TM5-VKFB-85 M CASTRO</v>
       </c>
       <c r="B8">
-        <v>6618</v>
+        <v>6609</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -987,10 +1001,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>GC MAXUS PCRF-25 TERRENO</v>
+        <v>GC TM5-VRVJ-20 L SALINAS</v>
       </c>
       <c r="B9">
-        <v>6617</v>
+        <v>6620</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1001,10 +1015,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>GC MAXUS PKFF-65 G VICENCIO</v>
+        <v>GLP ALJIBE SJHW-20</v>
       </c>
       <c r="B10">
-        <v>6616</v>
+        <v>6583</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -1015,10 +1029,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>GC TM5-VKFB-85 M CASTRO</v>
+        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
       </c>
       <c r="B11">
-        <v>6609</v>
+        <v>6593</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -1029,10 +1043,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>GC TM5-VRVJ-20 L SALINAS</v>
+        <v>GLP SHDV-51 J REBOLLEDO</v>
       </c>
       <c r="B12">
-        <v>6620</v>
+        <v>6598</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -1043,10 +1057,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>GLP DF6 SRSK-54 TOPOGRAFIA</v>
+        <v>GLP SHLC-75 L FONSECA</v>
       </c>
       <c r="B13">
-        <v>6593</v>
+        <v>6586</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -1057,10 +1071,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>GLP DF6 SRSL-99 EMERGENCIA</v>
+        <v>GLP SHXP-98 CAMION PLUMA</v>
       </c>
       <c r="B14">
-        <v>6597</v>
+        <v>6604</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -1071,10 +1085,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>GLP SHDV-51 J REBOLLEDO</v>
+        <v>GLP SHXP-99 ALZA HOMBRE</v>
       </c>
       <c r="B15">
-        <v>6598</v>
+        <v>6601</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -1085,10 +1099,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>GLP SHXP-98 CAMION PLUMA</v>
+        <v>GLP SKDX-44 V VIAL</v>
       </c>
       <c r="B16">
-        <v>6604</v>
+        <v>6606</v>
       </c>
       <c r="C16">
         <v>1</v>
@@ -1099,10 +1113,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>GLP SHXP-99 ALZA HOMBRE</v>
+        <v>GLP SSZD-71  J VALLEJOS</v>
       </c>
       <c r="B17">
-        <v>6601</v>
+        <v>6580</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -1113,10 +1127,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>GLP SSZD-71  J VALLEJOS</v>
+        <v>GLP TM5 TDKV-89 PAISAJISMO</v>
       </c>
       <c r="B18">
-        <v>6580</v>
+        <v>6594</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -1127,10 +1141,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>GLP TM5 TDKV-89 PAISAJISMO</v>
+        <v>GP -SHLC-76 F SEPULVEDA</v>
       </c>
       <c r="B19">
-        <v>6594</v>
+        <v>6605</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1141,10 +1155,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>GP -SHLC-76 F SEPULVEDA</v>
+        <v>GP CHANGAN RRDF-75 L LOBOS</v>
       </c>
       <c r="B20">
-        <v>6605</v>
+        <v>6603</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -1155,10 +1169,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>GP CHANGAN RRDF-75 L LOBOS</v>
+        <v>GP FOTON G7 TSVS-96</v>
       </c>
       <c r="B21">
-        <v>6603</v>
+        <v>6602</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -1169,10 +1183,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>GP FOTON G7 TSVS-96</v>
+        <v>GP TM5 TRRD-32 V PIZARRO</v>
       </c>
       <c r="B22">
-        <v>6602</v>
+        <v>6612</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -1183,10 +1197,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>GP TM5 TRRD-32 V PIZARRO</v>
+        <v>GP TM5 TSDK-95 L MUNOZ</v>
       </c>
       <c r="B23">
-        <v>6612</v>
+        <v>6599</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -1197,10 +1211,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>GP TM5 TSDK-95 L MUNOZ</v>
+        <v>GV FORD BU-9781 V OLIVARES</v>
       </c>
       <c r="B24">
-        <v>6599</v>
+        <v>6621</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -1323,21 +1337,35 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
+        <v>GV TOLVA SPGW-29 V OLIVARES</v>
+      </c>
+      <c r="B33">
+        <v>6619</v>
+      </c>
+      <c r="C33">
+        <v>1</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
         <v>JAC  LYTS-17 G GALEA</v>
       </c>
-      <c r="B33">
+      <c r="B34">
         <v>6614</v>
       </c>
-      <c r="C33">
-        <v>1</v>
-      </c>
-      <c r="D33">
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D34"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>